<commit_message>
Refine SQL prompt in OllamaRunner for improved schema awareness and clean output handling
</commit_message>
<xml_diff>
--- a/evals/reports/benchmark.xlsx
+++ b/evals/reports/benchmark.xlsx
@@ -542,20 +542,30 @@
           <t>SELECT name ,  country  FROM singer ORDER BY birthday ASC</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>```sql
+SELECT name, country
+FROM singers
+ORDER BY age DESC;
+```</t>
+        </is>
+      </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>0.7899999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>0.338</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.23</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1412,7 +1422,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SELECT COUNT(*) FROM Singers;</t>
+          <t>SELECT COUNT(*) FROM singer;</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -1428,7 +1438,7 @@
         <v>0.518</v>
       </c>
       <c r="I32" t="n">
-        <v>4.54</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -1449,11 +1459,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SELECT COUNT(*) AS Total_Singers FROM Singers;</t>
+          <t>SELECT COUNT(*) FROM singer;</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F33" t="n">
         <v>0.6</v>
@@ -1462,10 +1472,10 @@
         <v>0.4399999999999999</v>
       </c>
       <c r="H33" t="n">
-        <v>0.268</v>
+        <v>0.518</v>
       </c>
       <c r="I33" t="n">
-        <v>7.14</v>
+        <v>4.61</v>
       </c>
     </row>
     <row r="34">
@@ -1486,10 +1496,9 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SELECT s.name, c.country
-FROM singers s
-JOIN countries c ON s.country_id = c.id
-ORDER BY s.age DESC;</t>
+          <t>SELECT name, country 
+FROM singer 
+ORDER BY DATE_PART('year', age(birthday)) DESC;</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -1505,7 +1514,7 @@
         <v>0.268</v>
       </c>
       <c r="I34" t="n">
-        <v>13.19</v>
+        <v>11.85</v>
       </c>
     </row>
     <row r="35">
@@ -1526,9 +1535,9 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SELECT s.name, s.country, s.age
-FROM singers s
-ORDER BY s.age DESC;</t>
+          <t>SELECT s.name, s.country 
+FROM singer s 
+ORDER BY DATEDIFF(CURDATE(), s.birthday) DESC;</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -1544,7 +1553,7 @@
         <v>0.268</v>
       </c>
       <c r="I35" t="n">
-        <v>9.449999999999999</v>
+        <v>12.71</v>
       </c>
     </row>
     <row r="36">
@@ -1565,9 +1574,9 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>SELECT AVG(id), MIN(id), MAX(id)
-FROM singers
-WHERE country='France';</t>
+          <t>SELECT AVG(id), MIN(id), MAX(id) 
+FROM singer 
+WHERE country = 'France';</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -1583,7 +1592,7 @@
         <v>0.268</v>
       </c>
       <c r="I36" t="n">
-        <v>9.359999999999999</v>
+        <v>9.529999999999999</v>
       </c>
     </row>
     <row r="37">
@@ -1604,9 +1613,9 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>SELECT AVG(s.id), MIN(s.id), MAX(s.id)
-FROM singers s
-WHERE s.country = 'France';</t>
+          <t>SELECT AVG(id) AS avg_id, MIN(id) AS min_id, MAX(id) AS max_id 
+FROM singer 
+WHERE country='France';</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -1622,7 +1631,7 @@
         <v>0.268</v>
       </c>
       <c r="I37" t="n">
-        <v>9.26</v>
+        <v>11.46</v>
       </c>
     </row>
     <row r="38">
@@ -1643,10 +1652,10 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>SELECT s.name, s.release_year
-FROM singers s
-WHERE s.age = (SELECT MIN(age) FROM singers)
-ORDER BY s.name;</t>
+          <t>SELECT s.name, s.birthday AS birth_year 
+FROM singer s 
+WHERE (SELECT COUNT(*) FROM singer) = 
+       ROW_NUMBER() OVER (ORDER BY s.birthday ASC);</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -1662,7 +1671,7 @@
         <v>0.268</v>
       </c>
       <c r="I38" t="n">
-        <v>12.21</v>
+        <v>16.62</v>
       </c>
     </row>
     <row r="39">
@@ -1683,12 +1692,10 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>SELECT s.name, s.release_year
-FROM singers s
-JOIN songs sgn ON s.id = sgn.singer_id
-ORDER BY s.age ASC;
-SELECT * FROM singers WHERE age = (SELECT MIN(age) FROM singers);
-SELECT name, release_year FROM songs WHERE singer_id IN (SELECT id FROM singers ORDER BY age ASC LIMIT 1);</t>
+          <t>SELECT s.name, 'No year provided' AS release_year
+FROM singer s
+WHERE s.id IN (SELECT MIN(s2.id) 
+               FROM singer s2);</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -1704,7 +1711,7 @@
         <v>0.268</v>
       </c>
       <c r="I39" t="n">
-        <v>26.19</v>
+        <v>14.49</v>
       </c>
     </row>
     <row r="40">
@@ -1726,8 +1733,8 @@
       <c r="D40" t="inlineStr">
         <is>
           <t>SELECT DISTINCT country 
-FROM artists 
-WHERE birth_year = 2001;</t>
+FROM singer 
+WHERE YEAR(birthday) = 2001;</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -1743,7 +1750,7 @@
         <v>0.268</v>
       </c>
       <c r="I40" t="n">
-        <v>7.59</v>
+        <v>8.56</v>
       </c>
     </row>
     <row r="41">
@@ -1764,9 +1771,9 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>SELECT country 
-FROM singers 
-WHERE birth_year = 2001</t>
+          <t>SELECT DISTINCT country 
+FROM singer 
+WHERE YEAR(birthday) = 2001;</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -1782,7 +1789,7 @@
         <v>0.268</v>
       </c>
       <c r="I41" t="n">
-        <v>6.76</v>
+        <v>8.5</v>
       </c>
     </row>
   </sheetData>
@@ -1861,15 +1868,17 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.07899999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>0.0338</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.23</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1898,7 +1907,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="C5" t="n">
         <v>0.6</v>
@@ -1907,10 +1916,10 @@
         <v>0.4399999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>0.293</v>
+        <v>0.318</v>
       </c>
       <c r="F5" t="n">
-        <v>10.569</v>
+        <v>10.233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add evaluation reports for gemini_flash and ollama_llama3 models
- Created report_gemini_flash.json with evaluation metrics for various queries, all resulting in zero scores.
- Created report_ollama_llama3.json with evaluation metrics showing high accuracy and performance for various queries.
</commit_message>
<xml_diff>
--- a/evals/reports/benchmark.xlsx
+++ b/evals/reports/benchmark.xlsx
@@ -623,7 +623,7 @@
         <v>1</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0.2</v>
+        <v>0.49</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>1</v>
@@ -684,7 +684,7 @@
         <v>1</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>0.31</v>
+        <v>0.37</v>
       </c>
       <c r="N3" s="4" t="n">
         <v>1</v>
@@ -747,7 +747,7 @@
         <v>1</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0.23</v>
+        <v>0.61</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>1</v>
@@ -810,7 +810,7 @@
         <v>1</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0.39</v>
+        <v>0.41</v>
       </c>
       <c r="N5" s="4" t="n">
         <v>1</v>
@@ -873,7 +873,7 @@
         <v>1</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>1</v>
@@ -936,7 +936,7 @@
         <v>1</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="N7" s="4" t="n">
         <v>1</v>
@@ -1000,7 +1000,7 @@
         <v>1</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>0.41</v>
+        <v>0.61</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>1</v>
@@ -1032,7 +1032,8 @@
         <is>
           <t>SELECT name 
 FROM singer 
-WHERE birthday = (SELECT MAX(birthday) FROM singer)
+ORDER BY birthday DESC 
+LIMIT 1;
 ```</t>
         </is>
       </c>
@@ -1063,7 +1064,7 @@
         <v>1</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
       <c r="N9" s="4" t="n">
         <v>1</v>
@@ -1126,7 +1127,7 @@
         <v>1</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>1</v>
@@ -1189,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0.51</v>
+        <v>0.41</v>
       </c>
       <c r="N11" s="4" t="n">
         <v>1</v>
@@ -1283,7 +1284,7 @@
         <v>0.74</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.346</v>
+        <v>0.493</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(graph): Add extractor node for Phase 2 schema extraction
</commit_message>
<xml_diff>
--- a/evals/reports/benchmark.xlsx
+++ b/evals/reports/benchmark.xlsx
@@ -1011,8 +1011,8 @@
         <is>
           <t>SELECT name 
 FROM singer 
-ORDER BY birthday DESC 
-LIMIT 1</t>
+WHERE birthday = (SELECT MAX(birthday) FROM singer)
+```</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
@@ -1039,17 +1039,17 @@
         <v>1</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>0.85</v>
+        <v>0.45</v>
       </c>
       <c r="M9" s="4" t="n"/>
       <c r="N9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>0.315</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="10">
@@ -1428,7 +1428,7 @@
         <is>
           <t>SELECT AVG(id) AS average\_id, MIN(id) AS min\_id, MAX(id) AS max\_id
 FROM singer
-WHERE country = 'France' OR country = 'French';</t>
+WHERE country = 'France';</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
@@ -1486,14 +1486,9 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>SELECT
-    AVG(id) AS average_id,
-    MIN(id) AS minimum_id,
-    MAX(id) AS maximum_id
-FROM
-    singer
-WHERE
-    country = 'France' OR country = 'French';</t>
+          <t>SELECT AVG(id) AS average\_id, MIN(id) AS minimum\_id, MAX(id) AS maximum\_id
+FROM singer
+WHERE country IN ('France', 'French');</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
@@ -1520,17 +1515,17 @@
         <v>1</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0.85</v>
+        <v>0.45</v>
       </c>
       <c r="M17" s="4" t="n"/>
       <c r="N17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>0.315</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="18">
@@ -1551,9 +1546,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>SELECT name, MIN(birthday) AS "release year of the song"
+          <t>SELECT min(birthday) AS min_birthday
+    FROM singer
+)
+SELECT name
 FROM singer
-GROUP BY name;</t>
+JOIN young_singer ON singer.birthday = young_singer.min_birthday;</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -1580,17 +1578,17 @@
         <v>1</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>0.85</v>
+        <v>0.45</v>
       </c>
       <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>0.315</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="19">
@@ -1611,10 +1609,10 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>SELECT name, MIN(birthday) as "youngest_singer_birthday"
+          <t>SELECT name, MIN(birthday) AS youngest_birthday
 FROM singer
 GROUP BY name
-ORDER BY youngest_singer_birthday ASC
+ORDER BY youngest_birthday ASC
 LIMIT 1;</t>
         </is>
       </c>
@@ -1675,7 +1673,7 @@
         <is>
           <t>SELECT DISTINCT country
 FROM singer
-WHERE birthday = 2001;</t>
+WHERE EXTRACT(YEAR FROM birthday) = 2001;</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
@@ -1702,17 +1700,17 @@
         <v>1</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>0.85</v>
+        <v>0.45</v>
       </c>
       <c r="M20" s="2" t="n"/>
       <c r="N20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>0.315</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="21">
@@ -1848,13 +1846,13 @@
         <v>0.6</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.597</v>
+        <v>0.579</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0</v>
@@ -1873,13 +1871,13 @@
         <v>0.3</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.77</v>
+        <v>0.65</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.24</v>
+        <v>0.15</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.429</v>
+        <v>0.375</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Refactor graph builder and nodes for Phase 3 enhancements
- Updated graph_builder.py to implement a retry mechanism in the executor node, allowing it to attempt SQL execution up to MAX_RETRIES times on failure.
- Modified make_executor_node to accept a runner for generating correction prompts.
- Enhanced nodes.py to include a retry loop in the executor node while keeping the generator node unchanged.
- Added a failure/debug test injector in dataset_loader.py to facilitate testing of retry logic in Phase 3.
- Updated JSON reports to reflect changes in latency and execution results, including new test cases for error handling.
</commit_message>
<xml_diff>
--- a/evals/reports/benchmark.xlsx
+++ b/evals/reports/benchmark.xlsx
@@ -948,7 +948,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>SELECT name, EXTRACT(YEAR FROM birthday) 
+          <t>SELECT name, STRFTIME('%Y', birthday) 
 FROM singer 
 ORDER BY birthday DESC 
 LIMIT 1</t>
@@ -978,17 +978,17 @@
         <v>1</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0.45</v>
+        <v>0.85</v>
       </c>
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>0.135</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="9">
@@ -1306,8 +1306,8 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>SELECT name, country 
-FROM singer 
+          <t>SELECT name, country
+FROM singer
 ORDER BY birthday DESC;</t>
         </is>
       </c>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>SELECT AVG(id) AS average\_id, MIN(id) AS min\_id, MAX(id) AS max\_id
+          <t>SELECT AVG(id) AS average_id, MIN(id) AS min_id, MAX(id) AS max_id
 FROM singer
 WHERE country = 'France';</t>
         </is>
@@ -1455,17 +1455,17 @@
         <v>1</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>0.45</v>
+        <v>0.85</v>
       </c>
       <c r="M16" s="2" t="n"/>
       <c r="N16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>0.135</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="17">
@@ -1486,9 +1486,14 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>SELECT AVG(id) AS average\_id, MIN(id) AS minimum\_id, MAX(id) AS maximum\_id
-FROM singer
-WHERE country IN ('France', 'French');</t>
+          <t>SELECT
+    AVG(id) AS average_id,
+    MIN(id) AS minimum_id,
+    MAX(id) AS maximum_id
+FROM
+    singer
+WHERE
+    country IN ('France', 'French');</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
@@ -1515,17 +1520,17 @@
         <v>1</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0.45</v>
+        <v>0.85</v>
       </c>
       <c r="M17" s="4" t="n"/>
       <c r="N17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>0.135</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="18">
@@ -1546,12 +1551,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>SELECT min(birthday) AS min_birthday
+          <t>SELECT name
+FROM singer
+JOIN (
+    SELECT MIN(birthday) AS min_birthday
     FROM singer
-)
-SELECT name
-FROM singer
-JOIN young_singer ON singer.birthday = young_singer.min_birthday;</t>
+) AS young_singer ON singer.birthday = young_singer.min_birthday;</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -1578,17 +1583,17 @@
         <v>1</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>0.45</v>
+        <v>0.85</v>
       </c>
       <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>0.135</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="19">
@@ -1609,11 +1614,9 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>SELECT name, MIN(birthday) AS youngest_birthday
+          <t>SELECT name, birthday
 FROM singer
-GROUP BY name
-ORDER BY youngest_birthday ASC
-LIMIT 1;</t>
+WHERE id = (SELECT MIN(id) FROM singer);</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
@@ -1846,13 +1849,13 @@
         <v>0.6</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.24</v>
+        <v>0.27</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.579</v>
+        <v>0.597</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0</v>
@@ -1871,13 +1874,13 @@
         <v>0.3</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.65</v>
+        <v>0.77</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.15</v>
+        <v>0.24</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.375</v>
+        <v>0.429</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat: add lightweight experiment tracking and reproducibility layer
- Introduced ExperimentTracker class for tracking evaluation runs.
- Implemented methods to save configuration, results, and traces of the evaluation.
- Updated run_eval.py to initialize and utilize the ExperimentTracker for logging experiment details.
- Ensured all methods in ExperimentTracker are wrapped in try/except to prevent crashes.
- Stored experiment artifacts in evals/experiments/ directory for reproducibility.
</commit_message>
<xml_diff>
--- a/evals/reports/benchmark.xlsx
+++ b/evals/reports/benchmark.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -888,8 +888,8 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>SELECT AVG(id) AS average_id, MIN(id) AS min_id, MAX(id) AS max_id
-FROM singer
+          <t>SELECT AVG(id), MIN(id), MAX(id) 
+FROM singer 
 WHERE country = 'France'</t>
         </is>
       </c>
@@ -1132,17 +1132,17 @@
         <is>
           <t>SELECT DISTINCT country 
 FROM singer 
-WHERE birthday LIKE '2001%'</t>
+WHERE birthday BETWEEN '2001-01-01' AND '2001-12-31'</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4" t="n">
         <v>1</v>
@@ -1170,610 +1170,6 @@
       </c>
       <c r="P11" s="3" t="n">
         <v>0.8149999999999999</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>How many singers do we have?</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>SELECT count(*) FROM singer</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>SELECT COUNT(id) FROM singer;</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L12" s="2" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P12" s="3" t="n">
-        <v>0.8149999999999999</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>What is the total number of singers?</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>SELECT count(*) FROM singer</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>SELECT COUNT(id) FROM singer;</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" s="4" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="M13" s="4" t="n"/>
-      <c r="N13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P13" s="3" t="n">
-        <v>0.8149999999999999</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Show name, country for all singers ordered by age from the oldest to the youngest.</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>SELECT name ,  country  FROM singer ORDER BY birthday ASC</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>SELECT name, country
-FROM singer
-ORDER BY birthday DESC;</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L14" s="2" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P14" s="5" t="n">
-        <v>0.315</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>What are the names, countries for every singer in descending order of age?</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>SELECT name ,  country  FROM singer ORDER BY birthday ASC</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>SELECT name, country
-FROM singer
-ORDER BY birthday ASC;</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L15" s="4" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="M15" s="4" t="n"/>
-      <c r="N15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P15" s="3" t="n">
-        <v>0.8149999999999999</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>What is the average, minimum, and maximum id of all French singers?</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>SELECT avg(Singer_ID) ,  min(Singer_ID) ,  max(Singer_ID) FROM singer WHERE country  =  'France'</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>SELECT AVG(id) AS average_id, MIN(id) AS min_id, MAX(id) AS max_id
-FROM singer
-WHERE country = 'France';</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L16" s="2" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="M16" s="2" t="n"/>
-      <c r="N16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P16" s="5" t="n">
-        <v>0.315</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>What is the average, minimum, and maximum id for French singers?</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>SELECT avg(Singer_ID) ,  min(Singer_ID) ,  max(Singer_ID) FROM singer WHERE country  =  'France'</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>SELECT
-    AVG(id) AS average_id,
-    MIN(id) AS minimum_id,
-    MAX(id) AS maximum_id
-FROM
-    singer
-WHERE
-    country IN ('France', 'French');</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" s="4" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="M17" s="4" t="n"/>
-      <c r="N17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P17" s="5" t="n">
-        <v>0.315</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Show the name and the release year of the song by the youngest singer.</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>SELECT song_name ,  song_release_year FROM singer ORDER BY birthday desc LIMIT 1</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>SELECT name
-FROM singer
-JOIN (
-    SELECT MIN(birthday) AS min_birthday
-    FROM singer
-) AS young_singer ON singer.birthday = young_singer.min_birthday;</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="2" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P18" s="5" t="n">
-        <v>0.315</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>What are the names and release years for all the songs of the youngest singer?</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>SELECT song_name ,  song_release_year FROM singer ORDER BY birthday desc LIMIT 1</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>SELECT name, birthday
-FROM singer
-WHERE id = (SELECT MIN(id) FROM singer);</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" s="4" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="M19" s="4" t="n"/>
-      <c r="N19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P19" s="5" t="n">
-        <v>0.315</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>What are all distinct countries where singers born in 2001 are from?</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT country FROM singer WHERE birthday  like '2001%'</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT country
-FROM singer
-WHERE EXTRACT(YEAR FROM birthday) = 2001;</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="2" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="5" t="n">
-        <v>0.135</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>What are  the different countries with singers born in 2001?</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT country FROM singer WHERE birthday  like  '2001%'</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>SELECT DISTINCT country
-FROM singer
-WHERE EXTRACT(YEAR FROM birthday) = 2001;</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>single_agent</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L21" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="M21" s="4" t="n"/>
-      <c r="N21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="5" t="n">
-        <v>0.135</v>
       </c>
     </row>
   </sheetData>
@@ -1787,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1858,31 +1254,6 @@
         <v>0.597</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>multi_agent_groq_openrouter</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>0.429</v>
-      </c>
-      <c r="G3" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>